<commit_message>
EDDE 2026 Aggregators Changes
Potential fix for pull request finding

Co-authored-by: Copilot Autofix powered by AI <175728472+Copilot@users.noreply.github.com>

EDDE 2026 Aggregators Changes
</commit_message>
<xml_diff>
--- a/products/edde/resources/quality_of_life/transportation.xlsx
+++ b/products/edde/resources/quality_of_life/transportation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nyco365-my.sharepoint.com/personal/rlin_planning_nyc_gov/Documents/Desktop/Data Projects/EDDE/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexrichey/dev/data-engineering-de2/products/edde/resources/quality_of_life/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F00FE92E-A747-41C5-A7FA-1BF0CD3D4BDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2B3D827-5950-654E-B8DE-FCCB386FCCB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" firstSheet="3" activeTab="3" xr2:uid="{AAA3CD90-8A68-9346-81BF-A2EF630B06B2}"/>
+    <workbookView xWindow="-7620" yWindow="-26160" windowWidth="28800" windowHeight="17400" firstSheet="3" activeTab="3" xr2:uid="{AAA3CD90-8A68-9346-81BF-A2EF630B06B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Access_to_Jobs" sheetId="4" r:id="rId1"/>
@@ -76,7 +76,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -467,12 +467,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08E356E8-9B6B-324A-8DA7-4DB971FC9969}">
   <dimension ref="A1:B56"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -480,7 +480,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>4103</v>
       </c>
@@ -488,7 +488,7 @@
         <v>839695.92008562398</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>4104</v>
       </c>
@@ -496,7 +496,7 @@
         <v>1467537.90549093</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>4107</v>
       </c>
@@ -504,7 +504,7 @@
         <v>723925.27001636499</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4108</v>
       </c>
@@ -512,7 +512,7 @@
         <v>957704.16053066403</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>4109</v>
       </c>
@@ -520,7 +520,7 @@
         <v>227443.16377753299</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>4110</v>
       </c>
@@ -528,7 +528,7 @@
         <v>211165.37755442099</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>4111</v>
       </c>
@@ -536,7 +536,7 @@
         <v>342403.20993443899</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>4112</v>
       </c>
@@ -544,7 +544,7 @@
         <v>97663.457761439902</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>4121</v>
       </c>
@@ -552,7 +552,7 @@
         <v>1535999.89853525</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>4165</v>
       </c>
@@ -560,7 +560,7 @@
         <v>1519842.0544672201</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>4204</v>
       </c>
@@ -568,7 +568,7 @@
         <v>93004.732668417404</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>4205</v>
       </c>
@@ -576,7 +576,7 @@
         <v>79921.013198386107</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>4207</v>
       </c>
@@ -584,7 +584,7 @@
         <v>77242.842121920301</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>4208</v>
       </c>
@@ -592,7 +592,7 @@
         <v>46806.059561192596</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>4209</v>
       </c>
@@ -600,7 +600,7 @@
         <v>49247.743498495998</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>4210</v>
       </c>
@@ -608,7 +608,7 @@
         <v>26954.046348878499</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>4211</v>
       </c>
@@ -616,7 +616,7 @@
         <v>53136.528636255898</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>4212</v>
       </c>
@@ -624,7 +624,7 @@
         <v>27523.6475633265</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>4221</v>
       </c>
@@ -632,7 +632,7 @@
         <v>105980.272892129</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>4263</v>
       </c>
@@ -640,7 +640,7 @@
         <v>85553.686149979403</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>4301</v>
       </c>
@@ -648,7 +648,7 @@
         <v>259567.53387725199</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>4302</v>
       </c>
@@ -656,7 +656,7 @@
         <v>391342.93881286302</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>4303</v>
       </c>
@@ -664,7 +664,7 @@
         <v>121336.41346117</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>4304</v>
       </c>
@@ -672,7 +672,7 @@
         <v>91079.159879058701</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>4305</v>
       </c>
@@ -680,7 +680,7 @@
         <v>36130.686285746102</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>4306</v>
       </c>
@@ -688,7 +688,7 @@
         <v>148369.82680613501</v>
       </c>
     </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>4307</v>
       </c>
@@ -696,7 +696,7 @@
         <v>110039.59874824301</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>4308</v>
       </c>
@@ -704,7 +704,7 @@
         <v>108838.308030021</v>
       </c>
     </row>
-    <row r="30" spans="1:2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>4309</v>
       </c>
@@ -712,7 +712,7 @@
         <v>92986.253215654695</v>
       </c>
     </row>
-    <row r="31" spans="1:2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>4310</v>
       </c>
@@ -720,7 +720,7 @@
         <v>50260.657602867897</v>
       </c>
     </row>
-    <row r="32" spans="1:2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>4311</v>
       </c>
@@ -728,7 +728,7 @@
         <v>99719.252680961406</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>4312</v>
       </c>
@@ -736,7 +736,7 @@
         <v>126126.888796067</v>
       </c>
     </row>
-    <row r="34" spans="1:2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>4313</v>
       </c>
@@ -744,7 +744,7 @@
         <v>70801.452206542395</v>
       </c>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>4314</v>
       </c>
@@ -752,7 +752,7 @@
         <v>112459.30331992199</v>
       </c>
     </row>
-    <row r="36" spans="1:2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>4315</v>
       </c>
@@ -760,7 +760,7 @@
         <v>100236.800552489</v>
       </c>
     </row>
-    <row r="37" spans="1:2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>4316</v>
       </c>
@@ -768,7 +768,7 @@
         <v>57336.121867389404</v>
       </c>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>4317</v>
       </c>
@@ -776,7 +776,7 @@
         <v>65106.263583947701</v>
       </c>
     </row>
-    <row r="39" spans="1:2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>4318</v>
       </c>
@@ -784,7 +784,7 @@
         <v>43579.4844801867</v>
       </c>
     </row>
-    <row r="40" spans="1:2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>4401</v>
       </c>
@@ -792,7 +792,7 @@
         <v>173211.6124436</v>
       </c>
     </row>
-    <row r="41" spans="1:2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>4402</v>
       </c>
@@ -800,7 +800,7 @@
         <v>365418.14998793101</v>
       </c>
     </row>
-    <row r="42" spans="1:2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>4403</v>
       </c>
@@ -808,7 +808,7 @@
         <v>102982.02854154599</v>
       </c>
     </row>
-    <row r="43" spans="1:2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>4404</v>
       </c>
@@ -816,7 +816,7 @@
         <v>120054.47198785801</v>
       </c>
     </row>
-    <row r="44" spans="1:2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>4405</v>
       </c>
@@ -824,7 +824,7 @@
         <v>48198.704683167503</v>
       </c>
     </row>
-    <row r="45" spans="1:2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>4406</v>
       </c>
@@ -832,7 +832,7 @@
         <v>97002.139691160293</v>
       </c>
     </row>
-    <row r="46" spans="1:2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>4407</v>
       </c>
@@ -840,7 +840,7 @@
         <v>69905.946520284793</v>
       </c>
     </row>
-    <row r="47" spans="1:2">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>4408</v>
       </c>
@@ -848,7 +848,7 @@
         <v>65532.145598941097</v>
       </c>
     </row>
-    <row r="48" spans="1:2">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>4409</v>
       </c>
@@ -856,7 +856,7 @@
         <v>52236.525679758299</v>
       </c>
     </row>
-    <row r="49" spans="1:2">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>4410</v>
       </c>
@@ -864,7 +864,7 @@
         <v>27162.286728916901</v>
       </c>
     </row>
-    <row r="50" spans="1:2">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>4411</v>
       </c>
@@ -872,7 +872,7 @@
         <v>33605.554316528804</v>
       </c>
     </row>
-    <row r="51" spans="1:2">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>4412</v>
       </c>
@@ -880,7 +880,7 @@
         <v>39004.092989078097</v>
       </c>
     </row>
-    <row r="52" spans="1:2">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>4413</v>
       </c>
@@ -888,7 +888,7 @@
         <v>16846.260126047699</v>
       </c>
     </row>
-    <row r="53" spans="1:2">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>4414</v>
       </c>
@@ -896,7 +896,7 @@
         <v>12484.935255799701</v>
       </c>
     </row>
-    <row r="54" spans="1:2">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>4501</v>
       </c>
@@ -904,7 +904,7 @@
         <v>15823.534031786299</v>
       </c>
     </row>
-    <row r="55" spans="1:2">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>4502</v>
       </c>
@@ -912,7 +912,7 @@
         <v>13630.1853932177</v>
       </c>
     </row>
-    <row r="56" spans="1:2">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>4503</v>
       </c>
@@ -928,12 +928,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40868E50-81B0-CF42-B7D8-B81A3B0AF8C2}">
   <dimension ref="A1:D56"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="10.875" style="1"/>
+    <col min="4" max="4" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -947,7 +947,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>4103</v>
       </c>
@@ -961,7 +961,7 @@
         <v>0.27162393267173701</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>4104</v>
       </c>
@@ -975,7 +975,7 @@
         <v>0.36068541368506501</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>4107</v>
       </c>
@@ -989,7 +989,7 @@
         <v>0.68189620963175301</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4108</v>
       </c>
@@ -1003,7 +1003,7 @@
         <v>0.41606065961729899</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>4109</v>
       </c>
@@ -1017,7 +1017,7 @@
         <v>0.69819297832660299</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>4110</v>
       </c>
@@ -1031,7 +1031,7 @@
         <v>0.64262496166819905</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>4111</v>
       </c>
@@ -1045,7 +1045,7 @@
         <v>0.38148133423448399</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>4112</v>
       </c>
@@ -1059,7 +1059,7 @@
         <v>0.64512182203389801</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>4121</v>
       </c>
@@ -1073,7 +1073,7 @@
         <v>0.51899727188637901</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>4165</v>
       </c>
@@ -1087,7 +1087,7 @@
         <v>0.41856359539080501</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>4204</v>
       </c>
@@ -1101,7 +1101,7 @@
         <v>0.28939500933851597</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>4205</v>
       </c>
@@ -1115,7 +1115,7 @@
         <v>0.37010597586105298</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>4207</v>
       </c>
@@ -1129,7 +1129,7 @@
         <v>0.33483391454436501</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>4208</v>
       </c>
@@ -1143,7 +1143,7 @@
         <v>0.16290260679597299</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>4209</v>
       </c>
@@ -1157,7 +1157,7 @@
         <v>0.22737574137275099</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>4210</v>
       </c>
@@ -1171,7 +1171,7 @@
         <v>0.13513533976907</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>4211</v>
       </c>
@@ -1185,7 +1185,7 @@
         <v>0.33990018387181498</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>4212</v>
       </c>
@@ -1199,7 +1199,7 @@
         <v>0.24369638113486899</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>4221</v>
       </c>
@@ -1213,7 +1213,7 @@
         <v>0.43652270918332098</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>4263</v>
       </c>
@@ -1227,7 +1227,7 @@
         <v>0.10738715984557599</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>4301</v>
       </c>
@@ -1241,7 +1241,7 @@
         <v>0.33099326393141398</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>4302</v>
       </c>
@@ -1255,7 +1255,7 @@
         <v>0.53677242459851104</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>4303</v>
       </c>
@@ -1269,7 +1269,7 @@
         <v>0.29540042107200698</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>4304</v>
       </c>
@@ -1283,7 +1283,7 @@
         <v>0.411960545603617</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>4305</v>
       </c>
@@ -1297,7 +1297,7 @@
         <v>0.223787943396039</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>4306</v>
       </c>
@@ -1311,7 +1311,7 @@
         <v>0.32796390647247498</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>4307</v>
       </c>
@@ -1325,7 +1325,7 @@
         <v>0.31791393056407302</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>4308</v>
       </c>
@@ -1339,7 +1339,7 @@
         <v>0.43684573319240799</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>4309</v>
       </c>
@@ -1353,7 +1353,7 @@
         <v>0.46876716981508998</v>
       </c>
     </row>
-    <row r="31" spans="1:4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>4310</v>
       </c>
@@ -1367,7 +1367,7 @@
         <v>0.18562526522681</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>4311</v>
       </c>
@@ -1381,7 +1381,7 @@
         <v>0.47303389463397899</v>
       </c>
     </row>
-    <row r="33" spans="1:4">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>4312</v>
       </c>
@@ -1395,7 +1395,7 @@
         <v>0.323933622262773</v>
       </c>
     </row>
-    <row r="34" spans="1:4">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>4313</v>
       </c>
@@ -1409,7 +1409,7 @@
         <v>0.33862196014138202</v>
       </c>
     </row>
-    <row r="35" spans="1:4">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>4314</v>
       </c>
@@ -1423,7 +1423,7 @@
         <v>0.374853765162243</v>
       </c>
     </row>
-    <row r="36" spans="1:4">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>4315</v>
       </c>
@@ -1437,7 +1437,7 @@
         <v>0.18271485511017499</v>
       </c>
     </row>
-    <row r="37" spans="1:4">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>4316</v>
       </c>
@@ -1451,7 +1451,7 @@
         <v>0.29195357265292099</v>
       </c>
     </row>
-    <row r="38" spans="1:4">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>4317</v>
       </c>
@@ -1465,7 +1465,7 @@
         <v>0.21372540454185199</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>4318</v>
       </c>
@@ -1479,7 +1479,7 @@
         <v>1.36074202578559E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:4">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>4401</v>
       </c>
@@ -1493,7 +1493,7 @@
         <v>0.254119804590972</v>
       </c>
     </row>
-    <row r="41" spans="1:4">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>4402</v>
       </c>
@@ -1507,7 +1507,7 @@
         <v>0.42158656848648501</v>
       </c>
     </row>
-    <row r="42" spans="1:4">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>4403</v>
       </c>
@@ -1521,7 +1521,7 @@
         <v>0.21328450420731801</v>
       </c>
     </row>
-    <row r="43" spans="1:4">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>4404</v>
       </c>
@@ -1535,7 +1535,7 @@
         <v>0.30780828701920399</v>
       </c>
     </row>
-    <row r="44" spans="1:4">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>4405</v>
       </c>
@@ -1549,7 +1549,7 @@
         <v>0.12523564648008201</v>
       </c>
     </row>
-    <row r="45" spans="1:4">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>4406</v>
       </c>
@@ -1563,7 +1563,7 @@
         <v>0.24726413045294299</v>
       </c>
     </row>
-    <row r="46" spans="1:4">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>4407</v>
       </c>
@@ -1577,7 +1577,7 @@
         <v>2.3852878929464399E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:4">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>4408</v>
       </c>
@@ -1591,7 +1591,7 @@
         <v>5.6948084007443597E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:4">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>4409</v>
       </c>
@@ -1605,7 +1605,7 @@
         <v>0.222642155442597</v>
       </c>
     </row>
-    <row r="49" spans="1:4">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>4410</v>
       </c>
@@ -1619,7 +1619,7 @@
         <v>0.14232344773623401</v>
       </c>
     </row>
-    <row r="50" spans="1:4">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>4411</v>
       </c>
@@ -1633,7 +1633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:4">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>4412</v>
       </c>
@@ -1647,7 +1647,7 @@
         <v>8.8136592708693007E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:4">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>4413</v>
       </c>
@@ -1661,7 +1661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:4">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>4414</v>
       </c>
@@ -1675,7 +1675,7 @@
         <v>0.20443363637095599</v>
       </c>
     </row>
-    <row r="54" spans="1:4">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>4501</v>
       </c>
@@ -1689,7 +1689,7 @@
         <v>2.0376952527606899E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:4">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>4502</v>
       </c>
@@ -1703,7 +1703,7 @@
         <v>7.4178443545140499E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:4">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>4503</v>
       </c>
@@ -1725,9 +1725,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFAA854D-65E5-BC49-A74D-36D742BDC5CD}">
   <dimension ref="A1:D56"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1741,7 +1741,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>4103</v>
       </c>
@@ -1755,7 +1755,7 @@
         <v>0.81837183785804901</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>4104</v>
       </c>
@@ -1769,7 +1769,7 @@
         <v>0.56321510076199999</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>4107</v>
       </c>
@@ -1783,7 +1783,7 @@
         <v>0.71939414746810804</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4108</v>
       </c>
@@ -1797,7 +1797,7 @@
         <v>0.81003349383359902</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>4109</v>
       </c>
@@ -1811,7 +1811,7 @@
         <v>0.79453729019174701</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>4110</v>
       </c>
@@ -1825,7 +1825,7 @@
         <v>0.66182152713891396</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>4111</v>
       </c>
@@ -1839,7 +1839,7 @@
         <v>0.67685763129646503</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>4112</v>
       </c>
@@ -1853,7 +1853,7 @@
         <v>0.67051377118643996</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>4121</v>
       </c>
@@ -1867,7 +1867,7 @@
         <v>0.61658880419637696</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>4165</v>
       </c>
@@ -1881,7 +1881,7 @@
         <v>0.90874214238141704</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>4204</v>
       </c>
@@ -1895,7 +1895,7 @@
         <v>0.434475294179761</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>4205</v>
       </c>
@@ -1909,7 +1909,7 @@
         <v>0.47303503090962601</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>4207</v>
       </c>
@@ -1923,7 +1923,7 @@
         <v>0.61754905068864696</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>4208</v>
       </c>
@@ -1937,7 +1937,7 @@
         <v>0.16290260679597299</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>4209</v>
       </c>
@@ -1951,7 +1951,7 @@
         <v>0.34717943497618498</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>4210</v>
       </c>
@@ -1965,7 +1965,7 @@
         <v>0.14871853113761099</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>4211</v>
       </c>
@@ -1979,7 +1979,7 @@
         <v>0.38251083530338797</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>4212</v>
       </c>
@@ -1993,7 +1993,7 @@
         <v>0.270466153626019</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>4221</v>
       </c>
@@ -2007,7 +2007,7 @@
         <v>0.57559804714184504</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>4263</v>
       </c>
@@ -2021,7 +2021,7 @@
         <v>0.30818143046254898</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>4301</v>
       </c>
@@ -2035,7 +2035,7 @@
         <v>0.46564115125535799</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>4302</v>
       </c>
@@ -2049,7 +2049,7 @@
         <v>0.53677242459851104</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>4303</v>
       </c>
@@ -2063,7 +2063,7 @@
         <v>0.49725037677891398</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>4304</v>
       </c>
@@ -2077,7 +2077,7 @@
         <v>0.41956321896196103</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>4305</v>
       </c>
@@ -2091,7 +2091,7 @@
         <v>0.29158278874664001</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>4306</v>
       </c>
@@ -2105,7 +2105,7 @@
         <v>0.32796390647247498</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>4307</v>
       </c>
@@ -2119,7 +2119,7 @@
         <v>0.31791393056407302</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>4308</v>
       </c>
@@ -2133,7 +2133,7 @@
         <v>0.53441477873259502</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>4309</v>
       </c>
@@ -2147,7 +2147,7 @@
         <v>0.61013156448857597</v>
       </c>
     </row>
-    <row r="31" spans="1:4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>4310</v>
       </c>
@@ -2161,7 +2161,7 @@
         <v>0.21255369679643199</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>4311</v>
       </c>
@@ -2175,7 +2175,7 @@
         <v>0.60775612385217104</v>
       </c>
     </row>
-    <row r="33" spans="1:4">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>4312</v>
       </c>
@@ -2189,7 +2189,7 @@
         <v>0.323933622262773</v>
       </c>
     </row>
-    <row r="34" spans="1:4">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>4313</v>
       </c>
@@ -2203,7 +2203,7 @@
         <v>0.33862196014138202</v>
       </c>
     </row>
-    <row r="35" spans="1:4">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>4314</v>
       </c>
@@ -2217,7 +2217,7 @@
         <v>0.42943168524105602</v>
       </c>
     </row>
-    <row r="36" spans="1:4">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>4315</v>
       </c>
@@ -2231,7 +2231,7 @@
         <v>0.39738935046010798</v>
       </c>
     </row>
-    <row r="37" spans="1:4">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>4316</v>
       </c>
@@ -2245,7 +2245,7 @@
         <v>0.29195357265292099</v>
       </c>
     </row>
-    <row r="38" spans="1:4">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>4317</v>
       </c>
@@ -2259,7 +2259,7 @@
         <v>0.42278289847294398</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>4318</v>
       </c>
@@ -2273,7 +2273,7 @@
         <v>0.29295134644955201</v>
       </c>
     </row>
-    <row r="40" spans="1:4">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>4401</v>
       </c>
@@ -2287,7 +2287,7 @@
         <v>0.30714755661007798</v>
       </c>
     </row>
-    <row r="41" spans="1:4">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>4402</v>
       </c>
@@ -2301,7 +2301,7 @@
         <v>0.457460096146863</v>
       </c>
     </row>
-    <row r="42" spans="1:4">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>4403</v>
       </c>
@@ -2315,7 +2315,7 @@
         <v>0.27467501607447298</v>
       </c>
     </row>
-    <row r="43" spans="1:4">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>4404</v>
       </c>
@@ -2329,7 +2329,7 @@
         <v>0.37966763880482002</v>
       </c>
     </row>
-    <row r="44" spans="1:4">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>4405</v>
       </c>
@@ -2343,7 +2343,7 @@
         <v>0.142938414001584</v>
       </c>
     </row>
-    <row r="45" spans="1:4">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>4406</v>
       </c>
@@ -2357,7 +2357,7 @@
         <v>0.26885870382436899</v>
       </c>
     </row>
-    <row r="46" spans="1:4">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>4407</v>
       </c>
@@ -2371,7 +2371,7 @@
         <v>0.185508027908385</v>
       </c>
     </row>
-    <row r="47" spans="1:4">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>4408</v>
       </c>
@@ -2385,7 +2385,7 @@
         <v>0.209233729570974</v>
       </c>
     </row>
-    <row r="48" spans="1:4">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>4409</v>
       </c>
@@ -2399,7 +2399,7 @@
         <v>0.266388369459295</v>
       </c>
     </row>
-    <row r="49" spans="1:4">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>4410</v>
       </c>
@@ -2413,7 +2413,7 @@
         <v>0.19336749566578099</v>
       </c>
     </row>
-    <row r="50" spans="1:4">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>4411</v>
       </c>
@@ -2427,7 +2427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:4">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>4412</v>
       </c>
@@ -2441,7 +2441,7 @@
         <v>0.108911812972582</v>
       </c>
     </row>
-    <row r="52" spans="1:4">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>4413</v>
       </c>
@@ -2455,7 +2455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:4">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>4414</v>
       </c>
@@ -2469,7 +2469,7 @@
         <v>0.37587670207026502</v>
       </c>
     </row>
-    <row r="54" spans="1:4">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>4501</v>
       </c>
@@ -2483,7 +2483,7 @@
         <v>2.69319608070623E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:4">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>4502</v>
       </c>
@@ -2497,7 +2497,7 @@
         <v>0.178055102372325</v>
       </c>
     </row>
-    <row r="56" spans="1:4">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>4503</v>
       </c>
@@ -2519,27 +2519,27 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88B7800E-0291-1C4B-8F99-A30C41F8D597}">
   <dimension ref="A1:E56"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="10.875" style="3"/>
-    <col min="5" max="5" width="10.875" style="2"/>
+    <col min="4" max="4" width="10.83203125" style="3"/>
+    <col min="5" max="5" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
         <v>6</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>4103</v>
       </c>
@@ -2553,7 +2553,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>4104</v>
       </c>
@@ -2567,7 +2567,7 @@
         <v>0.95446563261517003</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>4107</v>
       </c>
@@ -2581,7 +2581,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4108</v>
       </c>
@@ -2595,7 +2595,7 @@
         <v>0.97611893974989505</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>4109</v>
       </c>
@@ -2609,7 +2609,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>4110</v>
       </c>
@@ -2623,7 +2623,7 @@
         <v>0.98199938669119902</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>4111</v>
       </c>
@@ -2637,7 +2637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>4112</v>
       </c>
@@ -2651,7 +2651,7 @@
         <v>0.99395127118644</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>4121</v>
       </c>
@@ -2665,7 +2665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>4165</v>
       </c>
@@ -2679,7 +2679,7 @@
         <v>0.92891877343600304</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>4204</v>
       </c>
@@ -2693,7 +2693,7 @@
         <v>0.99722814358216205</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>4205</v>
       </c>
@@ -2707,7 +2707,7 @@
         <v>0.99986753017368202</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>4207</v>
       </c>
@@ -2721,7 +2721,7 @@
         <v>0.98132375215752499</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>4208</v>
       </c>
@@ -2735,7 +2735,7 @@
         <v>0.92937344394256904</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>4209</v>
       </c>
@@ -2749,7 +2749,7 @@
         <v>0.89210648979088802</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>4210</v>
       </c>
@@ -2763,7 +2763,7 @@
         <v>0.60751845542305505</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>4211</v>
       </c>
@@ -2777,7 +2777,7 @@
         <v>0.92223207249802996</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>4212</v>
       </c>
@@ -2791,7 +2791,7 @@
         <v>0.74855201846448605</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>4221</v>
       </c>
@@ -2805,7 +2805,7 @@
         <v>0.97854112220404699</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>4263</v>
       </c>
@@ -2819,7 +2819,7 @@
         <v>0.994494386378868</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>4301</v>
       </c>
@@ -2833,7 +2833,7 @@
         <v>0.985518677281077</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>4302</v>
       </c>
@@ -2847,7 +2847,7 @@
         <v>0.98242068155111595</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>4303</v>
       </c>
@@ -2861,7 +2861,7 @@
         <v>0.91722943822551495</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>4304</v>
       </c>
@@ -2875,7 +2875,7 @@
         <v>0.87825784491540104</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>4305</v>
       </c>
@@ -2889,7 +2889,7 @@
         <v>0.81690483037653305</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>4306</v>
       </c>
@@ -2903,7 +2903,7 @@
         <v>0.93445182097335799</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>4307</v>
       </c>
@@ -2917,7 +2917,7 @@
         <v>0.84501069510717497</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>4308</v>
       </c>
@@ -2931,7 +2931,7 @@
         <v>0.90425991452598597</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>4309</v>
       </c>
@@ -2945,7 +2945,7 @@
         <v>0.888874459306913</v>
       </c>
     </row>
-    <row r="31" spans="1:4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>4310</v>
       </c>
@@ -2959,7 +2959,7 @@
         <v>0.90021515943388497</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>4311</v>
       </c>
@@ -2973,7 +2973,7 @@
         <v>0.62887163962584403</v>
       </c>
     </row>
-    <row r="33" spans="1:4">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>4312</v>
       </c>
@@ -2987,7 +2987,7 @@
         <v>0.72764598540145897</v>
       </c>
     </row>
-    <row r="34" spans="1:4">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>4313</v>
       </c>
@@ -3001,7 +3001,7 @@
         <v>0.93255237944134395</v>
       </c>
     </row>
-    <row r="35" spans="1:4">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>4314</v>
       </c>
@@ -3015,7 +3015,7 @@
         <v>0.600314020072655</v>
       </c>
     </row>
-    <row r="36" spans="1:4">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>4315</v>
       </c>
@@ -3029,7 +3029,7 @@
         <v>0.75702101866761295</v>
       </c>
     </row>
-    <row r="37" spans="1:4">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>4316</v>
       </c>
@@ -3043,7 +3043,7 @@
         <v>0.99634653998726597</v>
       </c>
     </row>
-    <row r="38" spans="1:4">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>4317</v>
       </c>
@@ -3057,7 +3057,7 @@
         <v>0.59064046479409305</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>4318</v>
       </c>
@@ -3071,7 +3071,7 @@
         <v>0.74841304262114094</v>
       </c>
     </row>
-    <row r="40" spans="1:4">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>4401</v>
       </c>
@@ -3085,7 +3085,7 @@
         <v>0.73033346975356295</v>
       </c>
     </row>
-    <row r="41" spans="1:4">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>4402</v>
       </c>
@@ -3099,7 +3099,7 @@
         <v>0.77008990167458202</v>
       </c>
     </row>
-    <row r="42" spans="1:4">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>4403</v>
       </c>
@@ -3113,7 +3113,7 @@
         <v>0.72959100947694999</v>
       </c>
     </row>
-    <row r="43" spans="1:4">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>4404</v>
       </c>
@@ -3127,7 +3127,7 @@
         <v>0.82590106201507696</v>
       </c>
     </row>
-    <row r="44" spans="1:4">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>4405</v>
       </c>
@@ -3141,7 +3141,7 @@
         <v>0.72807232813144895</v>
       </c>
     </row>
-    <row r="45" spans="1:4">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>4406</v>
       </c>
@@ -3155,7 +3155,7 @@
         <v>0.78085476083070104</v>
       </c>
     </row>
-    <row r="46" spans="1:4">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>4407</v>
       </c>
@@ -3169,7 +3169,7 @@
         <v>0.82038316780119802</v>
       </c>
     </row>
-    <row r="47" spans="1:4">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>4408</v>
       </c>
@@ -3183,7 +3183,7 @@
         <v>0.66749585406301803</v>
       </c>
     </row>
-    <row r="48" spans="1:4">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>4409</v>
       </c>
@@ -3197,7 +3197,7 @@
         <v>0.73496800021069797</v>
       </c>
     </row>
-    <row r="49" spans="1:4">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>4410</v>
       </c>
@@ -3211,7 +3211,7 @@
         <v>0.53572469660473399</v>
       </c>
     </row>
-    <row r="50" spans="1:4">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>4411</v>
       </c>
@@ -3225,7 +3225,7 @@
         <v>0.73267083993919802</v>
       </c>
     </row>
-    <row r="51" spans="1:4">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>4412</v>
       </c>
@@ -3239,7 +3239,7 @@
         <v>0.74998351172994904</v>
       </c>
     </row>
-    <row r="52" spans="1:4">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>4413</v>
       </c>
@@ -3253,7 +3253,7 @@
         <v>0.39293155954479803</v>
       </c>
     </row>
-    <row r="53" spans="1:4">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>4414</v>
       </c>
@@ -3267,7 +3267,7 @@
         <v>0.86819876476603797</v>
       </c>
     </row>
-    <row r="54" spans="1:4">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>4501</v>
       </c>
@@ -3281,7 +3281,7 @@
         <v>0.66242498391570703</v>
       </c>
     </row>
-    <row r="55" spans="1:4">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>4502</v>
       </c>
@@ -3295,7 +3295,7 @@
         <v>0.72469295364818298</v>
       </c>
     </row>
-    <row r="56" spans="1:4">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>4503</v>
       </c>
@@ -3326,6 +3326,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005035A9DB76FC71428FAF3BDB14932BCD" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1a354e4ef9d0763dce21aeadd2e9957b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3d51228c-8aff-4099-8ffe-73dfbb04b9a4" xmlns:ns3="4eab1d2f-0a6f-43b5-bd47-0cc182e7f81d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d918ddd34d575ac527de8456b2baa35f" ns2:_="" ns3:_="">
     <xsd:import namespace="3d51228c-8aff-4099-8ffe-73dfbb04b9a4"/>
@@ -3566,23 +3575,40 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BED9FD0F-6DBC-4DBF-82D5-CF98A5E34887}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BED9FD0F-6DBC-4DBF-82D5-CF98A5E34887}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3d51228c-8aff-4099-8ffe-73dfbb04b9a4"/>
+    <ds:schemaRef ds:uri="4eab1d2f-0a6f-43b5-bd47-0cc182e7f81d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD9DF012-7C7D-4469-A069-423F3A249169}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B3E7405-2A6A-4A6B-8D58-ED4EFE822097}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B3E7405-2A6A-4A6B-8D58-ED4EFE822097}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD9DF012-7C7D-4469-A069-423F3A249169}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3d51228c-8aff-4099-8ffe-73dfbb04b9a4"/>
+    <ds:schemaRef ds:uri="4eab1d2f-0a6f-43b5-bd47-0cc182e7f81d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>